<commit_message>
[stanley] updates the Lab6
</commit_message>
<xml_diff>
--- a/Labs/Lab6/DataAverage/120cm_average_data.xlsx
+++ b/Labs/Lab6/DataAverage/120cm_average_data.xlsx
@@ -1,40 +1,63 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stanley/Documents/COURSE/PROGRAMME/Python/Robotics-Group-15/Labs/Lab6/DataAverage/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{242F8D3A-FCA1-1C4E-A91D-4810299F6DFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+  <si>
+    <t>Angle</t>
+  </si>
+  <si>
+    <t>Distance / cm</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -46,93 +69,45 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -420,751 +395,743 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B92"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Angle</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Distance / cm</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2">
         <v>135</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2">
         <v>198.29</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3">
         <v>134</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3">
         <v>105.11</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4">
         <v>133</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4">
         <v>0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5">
         <v>132</v>
       </c>
-      <c r="B5" t="n">
-        <v>64.58</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
+      <c r="B5">
+        <v>264.58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6">
         <v>131</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6">
         <v>198.22</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="n">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7">
         <v>130</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7">
         <v>260.89</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="n">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8">
         <v>129</v>
       </c>
-      <c r="B8" t="n">
+      <c r="B8">
         <v>208.98</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="n">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9">
         <v>128</v>
       </c>
-      <c r="B9" t="n">
-        <v>158.39</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
+      <c r="B9">
+        <v>158.38999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10">
         <v>127</v>
       </c>
-      <c r="B10" t="n">
+      <c r="B10">
         <v>218.38</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="n">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11">
         <v>126</v>
       </c>
-      <c r="B11" t="n">
+      <c r="B11">
         <v>144.34</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="n">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12">
         <v>125</v>
       </c>
-      <c r="B12" t="n">
+      <c r="B12">
         <v>179.55</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="n">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13">
         <v>124</v>
       </c>
-      <c r="B13" t="n">
+      <c r="B13">
         <v>120.63</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="n">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14">
         <v>123</v>
       </c>
-      <c r="B14" t="n">
+      <c r="B14">
         <v>89.28</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="n">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15">
         <v>122</v>
       </c>
-      <c r="B15" t="n">
+      <c r="B15">
         <v>119.6</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="n">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16">
         <v>121</v>
       </c>
-      <c r="B16" t="n">
-        <v>98.54000000000001</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
+      <c r="B16">
+        <v>98.54</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17">
         <v>120</v>
       </c>
-      <c r="B17" t="n">
+      <c r="B17">
         <v>119.48</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="n">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18">
         <v>119</v>
       </c>
-      <c r="B18" t="n">
+      <c r="B18">
         <v>119.52</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="n">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19">
         <v>118</v>
       </c>
-      <c r="B19" t="n">
-        <v>76.65000000000001</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
+      <c r="B19">
+        <v>76.650000000000006</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20">
         <v>117</v>
       </c>
-      <c r="B20" t="n">
+      <c r="B20">
         <v>118.07</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="n">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21">
         <v>116</v>
       </c>
-      <c r="B21" t="n">
+      <c r="B21">
         <v>95.27</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="n">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22">
         <v>115</v>
       </c>
-      <c r="B22" t="n">
+      <c r="B22">
         <v>119.01</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="n">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23">
         <v>114</v>
       </c>
-      <c r="B23" t="n">
+      <c r="B23">
         <v>118.94</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="n">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24">
         <v>113</v>
       </c>
-      <c r="B24" t="n">
+      <c r="B24">
         <v>65.61</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="n">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25">
         <v>112</v>
       </c>
-      <c r="B25" t="n">
+      <c r="B25">
         <v>114.47</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="n">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26">
         <v>111</v>
       </c>
-      <c r="B26" t="n">
+      <c r="B26">
         <v>88.11</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="n">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27">
         <v>110</v>
       </c>
-      <c r="B27" t="n">
+      <c r="B27">
         <v>113.38</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="n">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28">
         <v>109</v>
       </c>
-      <c r="B28" t="n">
+      <c r="B28">
         <v>118.55</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="n">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29">
         <v>108</v>
       </c>
-      <c r="B29" t="n">
-        <v>90.79000000000001</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
+      <c r="B29">
+        <v>90.79</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30">
         <v>107</v>
       </c>
-      <c r="B30" t="n">
-        <v>98.79000000000001</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
+      <c r="B30">
+        <v>98.79</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31">
         <v>106</v>
       </c>
-      <c r="B31" t="n">
+      <c r="B31">
         <v>118.17</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="n">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32">
         <v>105</v>
       </c>
-      <c r="B32" t="n">
+      <c r="B32">
         <v>103.08</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="n">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33">
         <v>104</v>
       </c>
-      <c r="B33" t="n">
+      <c r="B33">
         <v>118.53</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="n">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34">
         <v>103</v>
       </c>
-      <c r="B34" t="n">
+      <c r="B34">
         <v>118.44</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="n">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35">
         <v>102</v>
       </c>
-      <c r="B35" t="n">
-        <v>83.25</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
+      <c r="B35" s="3">
+        <v>120.78</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36">
         <v>101</v>
       </c>
-      <c r="B36" t="n">
-        <v>102.21</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
+      <c r="B36">
+        <v>120.62</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37">
         <v>100</v>
       </c>
-      <c r="B37" t="n">
-        <v>57.14</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
+      <c r="B37" s="3">
+        <v>120.46</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38">
         <v>99</v>
       </c>
-      <c r="B38" t="n">
-        <v>78.58</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
+      <c r="B38">
+        <v>120.3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39">
         <v>98</v>
       </c>
-      <c r="B39" t="n">
-        <v>78.89</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
+      <c r="B39" s="3">
+        <v>120.14</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40">
         <v>97</v>
       </c>
-      <c r="B40" t="n">
-        <v>78.40000000000001</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
+      <c r="B40" s="3">
+        <v>119.98</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41">
         <v>96</v>
       </c>
-      <c r="B41" t="n">
-        <v>49.06</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
+      <c r="B41" s="3">
+        <v>119.82</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42">
         <v>95</v>
       </c>
-      <c r="B42" t="n">
-        <v>78.48999999999999</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
+      <c r="B42">
+        <v>119.66</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43">
         <v>94</v>
       </c>
-      <c r="B43" t="n">
-        <v>78.73</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
+      <c r="B43" s="3">
+        <v>119.5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44">
         <v>93</v>
       </c>
-      <c r="B44" t="n">
-        <v>64.56999999999999</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
+      <c r="B44">
+        <v>119.34</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45">
         <v>92</v>
       </c>
-      <c r="B45" t="n">
-        <v>47.92</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
+      <c r="B45" s="3">
+        <v>119.18</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46">
         <v>91</v>
       </c>
-      <c r="B46" t="n">
-        <v>77.98</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
+      <c r="B46">
+        <v>119.02</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" s="2">
         <v>90</v>
       </c>
-      <c r="B47" t="n">
-        <v>78.86</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
+      <c r="B47" s="2">
+        <v>118.86</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48">
         <v>89</v>
       </c>
-      <c r="B48" t="n">
-        <v>62.48</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
+      <c r="B48">
+        <v>119.32</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49">
         <v>88</v>
       </c>
-      <c r="B49" t="n">
-        <v>78.66</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
+      <c r="B49" s="3">
+        <v>119.78</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50">
         <v>87</v>
       </c>
-      <c r="B50" t="n">
-        <v>70.31</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
+      <c r="B50">
+        <v>120.24</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51">
         <v>86</v>
       </c>
-      <c r="B51" t="n">
-        <v>78.73</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
+      <c r="B51" s="3">
+        <v>120.7</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52">
         <v>85</v>
       </c>
-      <c r="B52" t="n">
-        <v>98.62</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
+      <c r="B52">
+        <v>121.16</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53">
         <v>84</v>
       </c>
-      <c r="B53" t="n">
+      <c r="B53">
         <v>118.12</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="n">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54">
         <v>83</v>
       </c>
-      <c r="B54" t="n">
+      <c r="B54">
         <v>75.36</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="n">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55">
         <v>82</v>
       </c>
-      <c r="B55" t="n">
+      <c r="B55">
         <v>116.17</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="n">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56">
         <v>81</v>
       </c>
-      <c r="B56" t="n">
-        <v>96.81999999999999</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n">
+      <c r="B56">
+        <v>96.82</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57">
         <v>80</v>
       </c>
-      <c r="B57" t="n">
+      <c r="B57">
         <v>118.33</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="n">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58">
         <v>79</v>
       </c>
-      <c r="B58" t="n">
+      <c r="B58">
         <v>106.56</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="n">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59">
         <v>78</v>
       </c>
-      <c r="B59" t="n">
+      <c r="B59">
         <v>103.7</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="n">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60">
         <v>77</v>
       </c>
-      <c r="B60" t="n">
+      <c r="B60">
         <v>92.27</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" t="n">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61">
         <v>76</v>
       </c>
-      <c r="B61" t="n">
+      <c r="B61">
         <v>118.52</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="n">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62">
         <v>75</v>
       </c>
-      <c r="B62" t="n">
+      <c r="B62">
         <v>102.81</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" t="n">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A63">
         <v>74</v>
       </c>
-      <c r="B63" t="n">
+      <c r="B63">
         <v>103.52</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" t="n">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A64">
         <v>73</v>
       </c>
-      <c r="B64" t="n">
+      <c r="B64">
         <v>92.3</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="n">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A65">
         <v>72</v>
       </c>
-      <c r="B65" t="n">
+      <c r="B65">
         <v>118.99</v>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="n">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A66">
         <v>71</v>
       </c>
-      <c r="B66" t="n">
+      <c r="B66">
         <v>100.27</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="n">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A67">
         <v>70</v>
       </c>
-      <c r="B67" t="n">
+      <c r="B67">
         <v>105.41</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="n">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68">
         <v>69</v>
       </c>
-      <c r="B68" t="n">
+      <c r="B68">
         <v>118.99</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" t="n">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69">
         <v>68</v>
       </c>
-      <c r="B69" t="n">
+      <c r="B69">
         <v>115.92</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="n">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70">
         <v>67</v>
       </c>
-      <c r="B70" t="n">
+      <c r="B70">
         <v>100.59</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="n">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71">
         <v>66</v>
       </c>
-      <c r="B71" t="n">
+      <c r="B71">
         <v>104.09</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" t="n">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A72">
         <v>65</v>
       </c>
-      <c r="B72" t="n">
+      <c r="B72">
         <v>119.52</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" t="n">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73">
         <v>64</v>
       </c>
-      <c r="B73" t="n">
+      <c r="B73">
         <v>107.88</v>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" t="n">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74">
         <v>63</v>
       </c>
-      <c r="B74" t="n">
-        <v>97.06999999999999</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="n">
+      <c r="B74">
+        <v>97.07</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75">
         <v>62</v>
       </c>
-      <c r="B75" t="n">
+      <c r="B75">
         <v>102.8</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" t="n">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A76">
         <v>61</v>
       </c>
-      <c r="B76" t="n">
+      <c r="B76">
         <v>120.01</v>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" t="n">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A77">
         <v>60</v>
       </c>
-      <c r="B77" t="n">
+      <c r="B77">
         <v>103.65</v>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" t="n">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A78">
         <v>59</v>
       </c>
-      <c r="B78" t="n">
-        <v>96.98999999999999</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="n">
+      <c r="B78">
+        <v>96.99</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A79">
         <v>58</v>
       </c>
-      <c r="B79" t="n">
+      <c r="B79">
         <v>99.55</v>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" t="n">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A80">
         <v>57</v>
       </c>
-      <c r="B80" t="n">
+      <c r="B80">
         <v>121.29</v>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" t="n">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A81">
         <v>56</v>
       </c>
-      <c r="B81" t="n">
-        <v>99.70999999999999</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="n">
+      <c r="B81">
+        <v>99.71</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A82">
         <v>55</v>
       </c>
-      <c r="B82" t="n">
+      <c r="B82">
         <v>105.69</v>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" t="n">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A83">
         <v>54</v>
       </c>
-      <c r="B83" t="n">
-        <v>142.89</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="n">
+      <c r="B83">
+        <v>142.88999999999999</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A84">
         <v>53</v>
       </c>
-      <c r="B84" t="n">
+      <c r="B84">
         <v>214.11</v>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" t="n">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A85">
         <v>52</v>
       </c>
-      <c r="B85" t="n">
+      <c r="B85">
         <v>190.42</v>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" t="n">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A86">
         <v>51</v>
       </c>
-      <c r="B86" t="n">
+      <c r="B86">
         <v>152.72</v>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" t="n">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A87">
         <v>50</v>
       </c>
-      <c r="B87" t="n">
+      <c r="B87">
         <v>94.67</v>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" t="n">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A88">
         <v>49</v>
       </c>
-      <c r="B88" t="n">
+      <c r="B88">
         <v>236.25</v>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" t="n">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A89">
         <v>48</v>
       </c>
-      <c r="B89" t="n">
+      <c r="B89">
         <v>200.04</v>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" t="n">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A90">
         <v>47</v>
       </c>
-      <c r="B90" t="n">
+      <c r="B90">
         <v>173.39</v>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" t="n">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A91">
         <v>46</v>
       </c>
-      <c r="B91" t="n">
+      <c r="B91">
         <v>142.54</v>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" t="n">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A92">
         <v>45</v>
       </c>
-      <c r="B92" t="n">
+      <c r="B92">
         <v>242.62</v>
       </c>
     </row>

</xml_diff>